<commit_message>
Lab 2 PHÂN VÙNG TƯƠNG ĐƯƠNG
</commit_message>
<xml_diff>
--- a/TESTER/Lab 2 PHÂN VÙNG TƯƠNG ĐƯƠNG.xlsx
+++ b/TESTER/Lab 2 PHÂN VÙNG TƯƠNG ĐƯƠNG.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TESTER\DangVanKhoa\TESTER\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0DD4215-BD9D-4D16-92D7-C3CC2597CE68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D278352F-BFAF-4D69-B03A-3FA4CAA3B552}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B04854CF-6AF7-4D59-B8A6-A60630F930F7}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{B04854CF-6AF7-4D59-B8A6-A60630F930F7}"/>
   </bookViews>
   <sheets>
     <sheet name="Bài 1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="152">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -302,9 +302,6 @@
     <t>Đặt xe lúc 8:00 PM</t>
   </si>
   <si>
-    <t xml:space="preserve">Kết quả </t>
-  </si>
-  <si>
     <t>X &lt; 40 cm</t>
   </si>
   <si>
@@ -492,6 +489,15 @@
   </si>
   <si>
     <t>Chứa chữ</t>
+  </si>
+  <si>
+    <t>Kết quả mong đợi</t>
+  </si>
+  <si>
+    <t>Kết quả thực tế</t>
+  </si>
+  <si>
+    <t>Failed</t>
   </si>
 </sst>
 </file>
@@ -524,7 +530,7 @@
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -549,8 +555,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -604,18 +616,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFDDDDDD"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFDDDDDD"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -639,23 +659,41 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="20" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -992,10 +1030,10 @@
       <c r="C1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="4"/>
+      <c r="E1" s="16"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
@@ -1021,7 +1059,7 @@
       <c r="A4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1035,7 +1073,7 @@
       <c r="C6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="5">
         <v>46174</v>
       </c>
       <c r="E6" s="3" t="s">
@@ -1046,175 +1084,193 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="28.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="B8" s="16"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
     </row>
     <row r="9" spans="1:6" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="8" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="22.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="10">
+      <c r="A10" s="9">
         <v>1</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="9" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="10">
+      <c r="A11" s="9">
         <v>2</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="D11" s="13">
+      <c r="D11" s="12">
         <v>0.03</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="11">
+      <c r="A12" s="10">
         <v>3</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="D12" s="12">
+      <c r="D12" s="11">
         <v>0.05</v>
       </c>
-      <c r="E12" s="11"/>
+      <c r="E12" s="10"/>
     </row>
     <row r="13" spans="1:6" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="11">
+      <c r="A13" s="10">
         <v>4</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D13" s="12">
+      <c r="D13" s="11">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="E13" s="11"/>
+      <c r="E13" s="10"/>
     </row>
     <row r="15" spans="1:6" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="19" t="s">
-        <v>108</v>
-      </c>
-      <c r="B15" s="19"/>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
+      <c r="A15" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="B15" s="18"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="18"/>
     </row>
     <row r="16" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="9" t="s">
+      <c r="A16" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="D16" s="9" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="7" t="s">
+      <c r="D16" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="E16" s="23" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C17" s="7">
+      <c r="C17" s="6">
         <v>-50</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="6" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="7" t="s">
+      <c r="E17" s="22" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="7">
+      <c r="C18" s="6">
         <v>0</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="6" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="7" t="s">
+      <c r="E18" s="22" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="7">
+      <c r="C19" s="6">
         <v>50</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="D19" s="6" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="7" t="s">
+      <c r="E19" s="22" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C20" s="7">
+      <c r="C20" s="6">
         <v>500</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="6" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="7" t="s">
+      <c r="E20" s="22" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C21" s="7">
+      <c r="C21" s="6">
         <v>1500</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="D21" s="6" t="s">
         <v>30</v>
+      </c>
+      <c r="E21" s="22" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -1237,6 +1293,7 @@
     <col min="2" max="2" width="15" customWidth="1"/>
     <col min="3" max="3" width="18.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
@@ -1249,10 +1306,10 @@
       <c r="C1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="E1" s="4"/>
+      <c r="E1" s="16"/>
       <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -1287,7 +1344,7 @@
       <c r="A4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>31</v>
       </c>
       <c r="C4" s="1"/>
@@ -1313,7 +1370,7 @@
       <c r="C6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="5">
         <v>46174</v>
       </c>
       <c r="E6" s="3" t="s">
@@ -1324,200 +1381,215 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="14"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
+      <c r="A7" s="13"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
     </row>
     <row r="8" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="B8" s="16"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
     </row>
     <row r="9" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="10"/>
-      <c r="B9" s="9" t="s">
+      <c r="A9" s="9"/>
+      <c r="B9" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="E9" s="10"/>
+      <c r="E9" s="9"/>
     </row>
     <row r="10" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="10"/>
-      <c r="B10" s="10" t="s">
+      <c r="A10" s="9"/>
+      <c r="B10" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E10" s="10"/>
+      <c r="E10" s="9"/>
     </row>
     <row r="11" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="10"/>
-      <c r="B11" s="10" t="s">
+      <c r="A11" s="9"/>
+      <c r="B11" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="E11" s="10"/>
+      <c r="E11" s="9"/>
     </row>
     <row r="12" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="10"/>
-      <c r="B12" s="10" t="s">
+      <c r="A12" s="9"/>
+      <c r="B12" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E12" s="10"/>
+      <c r="E12" s="9"/>
     </row>
     <row r="13" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="10"/>
-      <c r="B13" s="10" t="s">
+      <c r="A13" s="9"/>
+      <c r="B13" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E13" s="10"/>
+      <c r="E13" s="9"/>
     </row>
     <row r="14" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E14" s="15"/>
+      <c r="E14" s="14"/>
     </row>
     <row r="15" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="18" t="s">
+      <c r="A15" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="B15" s="18"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="10"/>
+      <c r="B15" s="19"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="9"/>
     </row>
     <row r="16" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="9" t="s">
+      <c r="A16" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="D16" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="E16" s="10"/>
+      <c r="D16" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="E16" s="23" t="s">
+        <v>150</v>
+      </c>
     </row>
     <row r="17" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="10" t="s">
+      <c r="A17" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="C17" s="10">
+      <c r="C17" s="9">
         <v>12345</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D17" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="E17" s="10"/>
+      <c r="E17" s="22" t="s">
+        <v>151</v>
+      </c>
     </row>
     <row r="18" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="10" t="s">
+      <c r="A18" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="C18" s="10">
+      <c r="C18" s="9">
         <v>123456</v>
       </c>
-      <c r="D18" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="E18" s="10"/>
+      <c r="D18" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E18" s="22" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="19" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="10" t="s">
+      <c r="A19" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="C19" s="10">
+      <c r="C19" s="9">
         <v>12345678</v>
       </c>
-      <c r="D19" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="E19" s="10"/>
+      <c r="D19" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E19" s="22" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="20" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="C20" s="10">
+      <c r="C20" s="9">
         <v>1234567890</v>
       </c>
-      <c r="D20" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="E20" s="10"/>
+      <c r="D20" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E20" s="22" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="21" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="10" t="s">
+      <c r="A21" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="10" t="s">
+      <c r="B21" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="C21" s="10">
+      <c r="C21" s="9">
         <v>12345678901</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D21" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="E21" s="10"/>
+      <c r="E21" s="22" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="22" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="10" t="s">
+      <c r="A22" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="C22" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="D22" s="9" t="s">
         <v>69</v>
+      </c>
+      <c r="E22" s="22" t="s">
+        <v>151</v>
       </c>
     </row>
   </sheetData>
@@ -1551,10 +1623,10 @@
       <c r="C1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="E1" s="4"/>
+      <c r="D1" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="E1" s="16"/>
       <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -1589,7 +1661,7 @@
       <c r="A4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>31</v>
       </c>
       <c r="C4" s="1"/>
@@ -1615,7 +1687,7 @@
       <c r="C6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="5">
         <v>46174</v>
       </c>
       <c r="E6" s="3" t="s">
@@ -1626,193 +1698,208 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="B8" s="16"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
     </row>
     <row r="9" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="10"/>
-      <c r="B9" s="9" t="s">
+      <c r="A9" s="9"/>
+      <c r="B9" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="E9" s="10"/>
+      <c r="E9" s="9"/>
     </row>
     <row r="10" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="10"/>
-      <c r="B10" s="10" t="s">
+      <c r="A10" s="9"/>
+      <c r="B10" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="E10" s="10"/>
+      <c r="E10" s="9"/>
     </row>
     <row r="11" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="10"/>
-      <c r="B11" s="10" t="s">
+      <c r="A11" s="9"/>
+      <c r="B11" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="E11" s="10"/>
+      <c r="E11" s="9"/>
     </row>
     <row r="12" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="10"/>
-      <c r="B12" s="10" t="s">
+      <c r="A12" s="9"/>
+      <c r="B12" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="E12" s="10"/>
+      <c r="E12" s="9"/>
     </row>
     <row r="13" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="10"/>
-      <c r="B13" s="10" t="s">
+      <c r="A13" s="9"/>
+      <c r="B13" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="E13" s="10"/>
+      <c r="E13" s="9"/>
     </row>
     <row r="14" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E14" s="15"/>
+      <c r="E14" s="14"/>
     </row>
     <row r="15" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="18" t="s">
+      <c r="A15" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="B15" s="18"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="10"/>
+      <c r="B15" s="19"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="9"/>
     </row>
     <row r="16" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="9" t="s">
+      <c r="A16" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="D16" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="E16" s="10"/>
+      <c r="D16" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="E16" s="24" t="s">
+        <v>150</v>
+      </c>
     </row>
     <row r="17" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="10" t="s">
+      <c r="A17" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="C17" s="17">
+      <c r="C17" s="15">
         <v>0.29166666666666669</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D17" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="E17" s="10"/>
+      <c r="E17" s="22" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="18" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="10" t="s">
+      <c r="A18" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="C18" s="17">
+      <c r="C18" s="15">
         <v>0.39583333333333331</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="D18" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E18" s="10"/>
+      <c r="E18" s="22" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="19" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="10" t="s">
+      <c r="A19" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="C19" s="17">
+      <c r="C19" s="15">
         <v>0.5</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E19" s="10"/>
+      <c r="E19" s="22" t="s">
+        <v>151</v>
+      </c>
     </row>
     <row r="20" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="C20" s="17">
+      <c r="C20" s="15">
         <v>0.66666666666666663</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="E20" s="10"/>
+      <c r="E20" s="22" t="s">
+        <v>151</v>
+      </c>
     </row>
     <row r="21" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="10" t="s">
+      <c r="A21" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="10" t="s">
+      <c r="B21" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="C21" s="17">
+      <c r="C21" s="15">
         <v>0.75</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D21" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="E21" s="15"/>
+      <c r="E21" s="22" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="22" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="10" t="s">
+      <c r="A22" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="C22" s="17">
+      <c r="C22" s="15">
         <v>0.83333333333333337</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="D22" s="9" t="s">
         <v>81</v>
+      </c>
+      <c r="E22" s="22" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -1833,7 +1920,7 @@
     <col min="2" max="2" width="13.6640625" customWidth="1"/>
     <col min="3" max="3" width="18.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
@@ -1846,10 +1933,10 @@
       <c r="C1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="E1" s="4"/>
+      <c r="D1" s="16" t="s">
+        <v>109</v>
+      </c>
+      <c r="E1" s="16"/>
       <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -1884,7 +1971,7 @@
       <c r="A4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>31</v>
       </c>
       <c r="C4" s="1"/>
@@ -1910,7 +1997,7 @@
       <c r="C6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="5">
         <v>46174</v>
       </c>
       <c r="E6" s="3" t="s">
@@ -1921,116 +2008,116 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="B8" s="16"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
     </row>
     <row r="9" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="10"/>
-      <c r="B9" s="9" t="s">
+      <c r="A9" s="9"/>
+      <c r="B9" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="8" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="42" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="10"/>
-      <c r="B10" s="10" t="s">
+      <c r="A10" s="9"/>
+      <c r="B10" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="9"/>
+      <c r="B11" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D11" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="9"/>
+      <c r="B12" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="9"/>
+      <c r="B13" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="9"/>
+      <c r="B14" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D14" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E14" s="9" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="10"/>
-      <c r="B11" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>88</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="10"/>
-      <c r="B12" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="D12" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="10"/>
-      <c r="B13" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="42" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="10"/>
-      <c r="B14" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="C14" s="10" t="s">
+    <row r="15" spans="1:6" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="9"/>
+      <c r="B15" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="C15" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D15" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E14" s="10" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="42" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="10"/>
-      <c r="B15" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>95</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="9" t="s">
         <v>38</v>
       </c>
     </row>
@@ -2044,124 +2131,140 @@
       <c r="E17" s="20"/>
     </row>
     <row r="18" spans="1:5" s="2" customFormat="1" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="9" t="s">
+      <c r="A18" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B18" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="D18" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="E18" s="10"/>
+      <c r="D18" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="E18" s="24" t="s">
+        <v>150</v>
+      </c>
     </row>
     <row r="19" spans="1:5" s="2" customFormat="1" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="C19" s="6">
+        <v>30</v>
+      </c>
+      <c r="D19" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="C19" s="7">
-        <v>30</v>
-      </c>
-      <c r="D19" s="7" t="s">
+      <c r="E19" s="22" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" s="2" customFormat="1" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="E19" s="7"/>
-    </row>
-    <row r="20" spans="1:5" s="2" customFormat="1" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="B20" s="7" t="s">
+      <c r="C20" s="6">
+        <v>70</v>
+      </c>
+      <c r="D20" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="C20" s="7">
-        <v>70</v>
-      </c>
-      <c r="D20" s="7" t="s">
+      <c r="E20" s="22" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" s="2" customFormat="1" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="E20" s="7"/>
-    </row>
-    <row r="21" spans="1:5" s="2" customFormat="1" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B21" s="7" t="s">
+      <c r="C21" s="6">
+        <v>120</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="E21" s="22" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" s="2" customFormat="1" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B22" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="C21" s="7">
-        <v>120</v>
-      </c>
-      <c r="D21" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="E21" s="7"/>
-    </row>
-    <row r="22" spans="1:5" s="2" customFormat="1" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="B22" s="7" t="s">
+      <c r="C22" s="6">
+        <v>170</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="E22" s="22" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" s="2" customFormat="1" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="C22" s="7">
-        <v>170</v>
-      </c>
-      <c r="D22" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="E22" s="7"/>
-    </row>
-    <row r="23" spans="1:5" s="2" customFormat="1" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B23" s="7" t="s">
+      <c r="C23" s="6">
+        <v>210</v>
+      </c>
+      <c r="D23" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="C23" s="7">
-        <v>210</v>
-      </c>
-      <c r="D23" s="7" t="s">
+      <c r="E23" s="22" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" s="2" customFormat="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="C24" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="E23" s="7"/>
-    </row>
-    <row r="24" spans="1:5" s="2" customFormat="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="B24" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="C24" s="7" t="s">
+      <c r="D24" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="E24" s="22" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" s="2" customFormat="1" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="D24" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="E24" s="7"/>
-    </row>
-    <row r="25" spans="1:5" s="2" customFormat="1" ht="28.2" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="7" t="s">
+      <c r="B25" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B25" s="7" t="s">
+      <c r="C25" s="6">
+        <v>-50</v>
+      </c>
+      <c r="D25" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="C25" s="7">
-        <v>-50</v>
-      </c>
-      <c r="D25" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="E25" s="8"/>
+      <c r="E25" s="7" t="s">
+        <v>151</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2194,10 +2297,10 @@
       <c r="C1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="E1" s="4"/>
+      <c r="D1" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="E1" s="16"/>
       <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -2232,7 +2335,7 @@
       <c r="A4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>31</v>
       </c>
       <c r="C4" s="1"/>
@@ -2258,7 +2361,7 @@
       <c r="C6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="5">
         <v>46174</v>
       </c>
       <c r="E6" s="3" t="s">
@@ -2269,233 +2372,252 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="B8" s="16"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="15"/>
-    </row>
-    <row r="9" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="9" t="s">
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="14"/>
+    </row>
+    <row r="9" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="E9" s="10"/>
-    </row>
-    <row r="10" spans="1:6" ht="42" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="10">
+      <c r="E9" s="9"/>
+    </row>
+    <row r="10" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="9">
         <v>1</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" s="9"/>
+    </row>
+    <row r="11" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="9">
+        <v>2</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D11" s="12">
+        <v>0.5</v>
+      </c>
+      <c r="E11" s="9"/>
+    </row>
+    <row r="12" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="9">
+        <v>3</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="D12" s="12">
+        <v>0.7</v>
+      </c>
+      <c r="E12" s="9"/>
+    </row>
+    <row r="13" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="9">
+        <v>4</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="D13" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E10" s="10"/>
-    </row>
-    <row r="11" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="10">
-        <v>2</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>113</v>
-      </c>
-      <c r="D11" s="13">
-        <v>0.5</v>
-      </c>
-      <c r="E11" s="10"/>
-    </row>
-    <row r="12" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="10">
-        <v>3</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>114</v>
-      </c>
-      <c r="D12" s="13">
-        <v>0.7</v>
-      </c>
-      <c r="E12" s="10"/>
-    </row>
-    <row r="13" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="10">
-        <v>4</v>
-      </c>
-      <c r="B13" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="C13" s="10" t="s">
+      <c r="E13" s="9"/>
+    </row>
+    <row r="14" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E14" s="14"/>
+    </row>
+    <row r="15" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="B15" s="17"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="9"/>
+    </row>
+    <row r="16" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="E16" s="24" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="D13" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="E13" s="10"/>
-    </row>
-    <row r="14" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E14" s="15"/>
-    </row>
-    <row r="15" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="21"/>
-      <c r="E15" s="10"/>
-    </row>
-    <row r="16" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B16" s="9" t="s">
+      <c r="C17" s="9">
         <v>15</v>
       </c>
-      <c r="C16" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D16" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="E16" s="10"/>
-    </row>
-    <row r="17" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="B17" s="10" t="s">
+      <c r="D17" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="C17" s="10">
-        <v>15</v>
-      </c>
-      <c r="D17" s="10" t="s">
+      <c r="E17" s="22" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="E17" s="10"/>
-    </row>
-    <row r="18" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="10" t="s">
+      <c r="C18" s="9">
         <v>20</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="D18" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="C18" s="10">
-        <v>20</v>
-      </c>
-      <c r="D18" s="10" t="s">
+      <c r="E18" s="22" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="E18" s="10"/>
-    </row>
-    <row r="19" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="B19" s="10" t="s">
+      <c r="C19" s="9">
+        <v>23</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="E19" s="22" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="C19" s="10">
-        <v>23</v>
-      </c>
-      <c r="D19" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="E19" s="10"/>
-    </row>
-    <row r="20" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="10" t="s">
+      <c r="C20" s="9">
         <v>25</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="D20" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="E20" s="22" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="C20" s="10">
-        <v>25</v>
-      </c>
-      <c r="D20" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="E20" s="10"/>
-    </row>
-    <row r="21" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="10" t="s">
+      <c r="C21" s="9">
+        <v>26</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="E21" s="22" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="C22" s="9">
         <v>28</v>
       </c>
-      <c r="B21" s="10" t="s">
+      <c r="D22" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="C21" s="10">
-        <v>26</v>
-      </c>
-      <c r="D21" s="10" t="s">
-        <v>123</v>
-      </c>
-      <c r="E21" s="10"/>
-    </row>
-    <row r="22" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="B22" s="10" t="s">
+      <c r="E22" s="9" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="B23" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="C22" s="10">
-        <v>28</v>
-      </c>
-      <c r="D22" s="10" t="s">
-        <v>123</v>
-      </c>
-      <c r="E22" s="10"/>
-    </row>
-    <row r="23" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="B23" s="10" t="s">
+      <c r="C23" s="9">
+        <v>30</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="E23" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="C23" s="10">
-        <v>30</v>
-      </c>
-      <c r="D23" s="10" t="s">
-        <v>123</v>
-      </c>
-      <c r="E23" s="15"/>
-    </row>
-    <row r="24" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="10" t="s">
+      <c r="B24" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="B24" s="10" t="s">
+      <c r="C24" s="9">
+        <v>35</v>
+      </c>
+      <c r="D24" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="C24" s="10">
-        <v>35</v>
-      </c>
-      <c r="D24" s="10" t="s">
-        <v>128</v>
+      <c r="E24" s="25" t="s">
+        <v>151</v>
       </c>
     </row>
   </sheetData>
@@ -2517,7 +2639,7 @@
     <col min="2" max="2" width="13.6640625" customWidth="1"/>
     <col min="3" max="3" width="18.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17.33203125" customWidth="1"/>
-    <col min="5" max="5" width="7.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
@@ -2530,10 +2652,10 @@
       <c r="C1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="E1" s="4"/>
+      <c r="D1" s="16" t="s">
+        <v>128</v>
+      </c>
+      <c r="E1" s="16"/>
       <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -2568,7 +2690,7 @@
       <c r="A4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>31</v>
       </c>
       <c r="C4" s="1"/>
@@ -2594,7 +2716,7 @@
       <c r="C6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="5">
         <v>46174</v>
       </c>
       <c r="E6" s="3" t="s">
@@ -2605,291 +2727,314 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="B8" s="16"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="15"/>
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="14"/>
     </row>
     <row r="9" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="E9" s="10"/>
+      <c r="E9" s="9"/>
     </row>
     <row r="10" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="10">
+      <c r="A10" s="9">
         <v>1</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" s="9"/>
+    </row>
+    <row r="11" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="9">
+        <v>2</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D11" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="E11" s="9"/>
+    </row>
+    <row r="12" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="9">
+        <v>3</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D12" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E10" s="10"/>
-    </row>
-    <row r="11" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="10">
-        <v>2</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>131</v>
-      </c>
-      <c r="D11" s="10" t="s">
+      <c r="E12" s="9"/>
+    </row>
+    <row r="13" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="9">
+        <v>4</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="D13" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="E11" s="10"/>
-    </row>
-    <row r="12" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="10">
-        <v>3</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="D12" s="10" t="s">
+      <c r="E13" s="9"/>
+    </row>
+    <row r="14" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="9">
+        <v>5</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="D14" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E12" s="10"/>
-    </row>
-    <row r="13" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="10">
-        <v>4</v>
-      </c>
-      <c r="B13" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="E13" s="10"/>
-    </row>
-    <row r="14" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="10">
-        <v>5</v>
-      </c>
-      <c r="B14" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="C14" s="10" t="s">
+      <c r="E14" s="9"/>
+    </row>
+    <row r="15" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="9">
+        <v>6</v>
+      </c>
+      <c r="B15" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="C15" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="D15" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E14" s="10"/>
-    </row>
-    <row r="15" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="10">
-        <v>6</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>135</v>
-      </c>
-      <c r="C15" s="10" t="s">
+      <c r="E15" s="9"/>
+    </row>
+    <row r="16" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E16" s="14"/>
+    </row>
+    <row r="17" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="9"/>
+    </row>
+    <row r="18" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="E18" s="24" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="D15" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="E15" s="10"/>
-    </row>
-    <row r="16" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E16" s="15"/>
-    </row>
-    <row r="17" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="B17" s="16"/>
-      <c r="C17" s="16"/>
-      <c r="D17" s="21"/>
-      <c r="E17" s="10"/>
-    </row>
-    <row r="18" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B18" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D18" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="E18" s="10"/>
-    </row>
-    <row r="19" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="B19" s="10" t="s">
+      <c r="C19" s="9"/>
+      <c r="D19" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10" t="s">
+      <c r="E19" s="22" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="E19" s="10"/>
-    </row>
-    <row r="20" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="B20" s="10" t="s">
+      <c r="C20" s="9">
+        <v>1</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E20" s="22" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="C20" s="10">
-        <v>1</v>
-      </c>
-      <c r="D20" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="E20" s="10"/>
-    </row>
-    <row r="21" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="B21" s="10" t="s">
+      <c r="C21" s="9">
+        <v>12345</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E21" s="22" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B22" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="C21" s="10">
-        <v>12345</v>
-      </c>
-      <c r="D21" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="E21" s="10"/>
-    </row>
-    <row r="22" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="B22" s="10" t="s">
+      <c r="C22" s="9">
+        <v>1234567890</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E22" s="22" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="C22" s="10">
-        <v>1234567890</v>
-      </c>
-      <c r="D22" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="E22" s="10"/>
-    </row>
-    <row r="23" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="B23" s="10" t="s">
+      <c r="C23" s="9">
+        <v>123456789012345</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="E23" s="22" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B24" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="C23" s="10">
-        <v>123456789012345</v>
-      </c>
-      <c r="D23" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="E23" s="10"/>
-    </row>
-    <row r="24" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="B24" s="10" t="s">
+      <c r="C24" s="9">
+        <v>1.23456789012345E+19</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E24" s="9" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="B25" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="C24" s="10">
-        <v>1.23456789012345E+19</v>
-      </c>
-      <c r="D24" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="E24" s="10"/>
-    </row>
-    <row r="25" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="B25" s="10" t="s">
+      <c r="C25" s="9">
+        <v>1.2345678901234501E+24</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E25" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="B26" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="C25" s="10">
-        <v>1.2345678901234501E+24</v>
-      </c>
-      <c r="D25" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="E25" s="10"/>
-    </row>
-    <row r="26" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="10" t="s">
-        <v>126</v>
-      </c>
-      <c r="B26" s="10" t="s">
+      <c r="C26" s="9">
+        <v>1.2345678901234499E+29</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E26" s="25" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="C26" s="10">
-        <v>1.2345678901234499E+29</v>
-      </c>
-      <c r="D26" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="E26" s="10"/>
-    </row>
-    <row r="27" spans="1:5" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="10" t="s">
+      <c r="B27" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="B27" s="10" t="s">
+      <c r="C27" s="9">
+        <v>1.23456789012345E+34</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="E27" s="14" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="C27" s="10">
-        <v>1.23456789012345E+34</v>
-      </c>
-      <c r="D27" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="E27" s="15"/>
-    </row>
-    <row r="28" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="10" t="s">
+      <c r="B28" s="9" t="s">
         <v>148</v>
       </c>
-      <c r="B28" s="10" t="s">
-        <v>149</v>
-      </c>
-      <c r="C28" s="10" t="s">
+      <c r="C28" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="D28" s="10" t="s">
+      <c r="D28" s="9" t="s">
         <v>69</v>
+      </c>
+      <c r="E28" s="26" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>